<commit_message>
data: publish 2026-10-01 sampler-linked operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-10-01-182路.xlsx
+++ b/data/export/2026-10-01-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC9"/>
+  <dimension ref="A1:AC15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -441,7 +441,7 @@
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
     <col width="26" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
@@ -665,7 +665,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -704,7 +704,7 @@
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA2" s="2" t="inlineStr">
@@ -715,7 +715,7 @@
       <c r="AB2" s="2" t="inlineStr"/>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/10</t>
         </is>
       </c>
     </row>
@@ -743,32 +743,36 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:32</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>72分钟</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -776,7 +780,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -800,33 +804,37 @@
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA3" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA3" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AB3" s="2" t="inlineStr">
+        <is>
+          <t>72.0</t>
+        </is>
+      </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>1/10</t>
         </is>
       </c>
     </row>
@@ -854,32 +862,36 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:49</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>74分钟</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -887,7 +899,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -911,17 +923,17 @@
       </c>
       <c r="W4" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y4" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z4" s="2" t="inlineStr">
@@ -931,13 +943,17 @@
       </c>
       <c r="AA4" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB4" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB4" s="2" t="inlineStr">
+        <is>
+          <t>74.0</t>
+        </is>
+      </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>2/10</t>
         </is>
       </c>
     </row>
@@ -965,32 +981,36 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>07:49</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>74分钟</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N5" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -998,7 +1018,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1022,33 +1042,37 @@
       </c>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y5" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA5" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA5" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB5" s="2" t="inlineStr"/>
+      <c r="AB5" s="2" t="inlineStr">
+        <is>
+          <t>74.0</t>
+        </is>
+      </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>2/10</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1133,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1148,7 +1172,7 @@
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA6" s="2" t="inlineStr">
@@ -1159,7 +1183,7 @@
       <c r="AB6" s="2" t="inlineStr"/>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/10</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1201,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>06:55</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -1220,7 +1244,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1234,7 +1258,7 @@
       <c r="T7" s="2" t="inlineStr"/>
       <c r="U7" s="2" t="inlineStr">
         <is>
-          <t>07:00</t>
+          <t>06:55</t>
         </is>
       </c>
       <c r="V7" s="2" t="inlineStr">
@@ -1270,7 +1294,7 @@
       <c r="AB7" s="2" t="inlineStr"/>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/10</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1355,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1381,7 +1405,7 @@
       <c r="AB8" s="2" t="inlineStr"/>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/10</t>
         </is>
       </c>
     </row>
@@ -1389,22 +1413,22 @@
       <c r="A9" s="2" t="inlineStr"/>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>沪A35717D</t>
+          <t>沪A13735A</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
           <t>金杨路金口路</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>07:25</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>川沙客运站</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -1437,12 +1461,12 @@
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>06:02</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>06:22</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1456,7 +1480,7 @@
       <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr">
         <is>
-          <t>07:25</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="V9" s="2" t="inlineStr">
@@ -1492,7 +1516,681 @@
       <c r="AB9" s="2" t="inlineStr"/>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>—/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>沪A35717D</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="inlineStr"/>
+      <c r="S10" s="2" t="inlineStr"/>
+      <c r="T10" s="2" t="inlineStr"/>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W10" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X10" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y10" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z10" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA10" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB10" s="2" t="inlineStr"/>
+      <c r="AC10" s="2" t="inlineStr">
+        <is>
+          <t>—/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>沪A68870D</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z11" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA11" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB11" s="2" t="inlineStr"/>
+      <c r="AC11" s="2" t="inlineStr">
+        <is>
+          <t>—/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>沪A55712D</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>07:45</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>07:45</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y12" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA12" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB12" s="2" t="inlineStr">
+        <is>
+          <t>72.0</t>
+        </is>
+      </c>
+      <c r="AC12" s="2" t="inlineStr">
+        <is>
+          <t>1/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>沪A67353D</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>07:50</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>07:11</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>07:50</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y13" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB13" s="2" t="inlineStr"/>
+      <c r="AC13" s="2" t="inlineStr">
+        <is>
+          <t>—/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>沪A67026D</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="inlineStr">
+        <is>
+          <t>74.0</t>
+        </is>
+      </c>
+      <c r="AC14" s="2" t="inlineStr">
+        <is>
+          <t>2/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>沪A67983D</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB15" s="2" t="inlineStr"/>
+      <c r="AC15" s="2" t="inlineStr">
+        <is>
+          <t>—/10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: publish 2026-10-01 rolling operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-10-01-182路.xlsx
+++ b/data/export/2026-10-01-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC22"/>
+  <dimension ref="A1:AC27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -665,7 +665,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -709,13 +709,17 @@
       </c>
       <c r="AA2" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB2" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB2" s="2" t="inlineStr">
+        <is>
+          <t>68.0</t>
+        </is>
+      </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>—/10</t>
+          <t>1/10</t>
         </is>
       </c>
     </row>
@@ -780,7 +784,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -834,7 +838,7 @@
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>4/10</t>
+          <t>5/10</t>
         </is>
       </c>
     </row>
@@ -899,7 +903,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -938,22 +942,22 @@
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA4" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AA4" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
-          <t>68.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>1/10</t>
+          <t>3/10</t>
         </is>
       </c>
     </row>
@@ -1018,7 +1022,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1057,7 +1061,7 @@
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA5" s="2" t="inlineStr">
@@ -1137,7 +1141,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1176,14 +1180,14 @@
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA6" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AA6" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
           <t>73.0</t>
@@ -1191,7 +1195,7 @@
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>5/10</t>
+          <t>6/10</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1256,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1291,7 +1295,7 @@
       </c>
       <c r="Z7" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA7" s="2" t="inlineStr">
@@ -1367,7 +1371,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1486,7 +1490,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1540,7 +1544,7 @@
       </c>
       <c r="AC9" s="2" t="inlineStr">
         <is>
-          <t>6/10</t>
+          <t>7/10</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1605,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1679,32 +1683,36 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>08:43</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>68分钟</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr"/>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr"/>
+          <t>SHMAAS终点近站ETA直接确认，约±2分钟</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -1712,7 +1720,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1736,17 +1744,17 @@
       </c>
       <c r="W11" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X11" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y11" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z11" s="2" t="inlineStr">
@@ -1756,13 +1764,17 @@
       </c>
       <c r="AA11" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB11" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB11" s="2" t="inlineStr">
+        <is>
+          <t>68.0</t>
+        </is>
+      </c>
       <c r="AC11" s="2" t="inlineStr">
         <is>
-          <t>—/10</t>
+          <t>1/10</t>
         </is>
       </c>
     </row>
@@ -1823,7 +1835,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1877,7 +1889,7 @@
       </c>
       <c r="AC12" s="2" t="inlineStr">
         <is>
-          <t>4/10</t>
+          <t>5/10</t>
         </is>
       </c>
     </row>
@@ -1905,32 +1917,36 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>09:05</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>75分钟</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr"/>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr"/>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
           <t>07:11</t>
@@ -1938,7 +1954,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -1962,33 +1978,37 @@
       </c>
       <c r="W13" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X13" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y13" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z13" s="2" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA13" s="2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB13" s="2" t="inlineStr"/>
+      <c r="AB13" s="2" t="inlineStr">
+        <is>
+          <t>75.0</t>
+        </is>
+      </c>
       <c r="AC13" s="2" t="inlineStr">
         <is>
-          <t>—/10</t>
+          <t>8/10</t>
         </is>
       </c>
     </row>
@@ -2049,7 +2069,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -2088,7 +2108,7 @@
       </c>
       <c r="Z14" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA14" s="2" t="inlineStr">
@@ -2131,32 +2151,36 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>09:20</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>70分钟</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N15" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -2164,7 +2188,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -2188,37 +2212,37 @@
       </c>
       <c r="W15" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X15" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y15" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z15" s="2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AA15" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
-          <t>68.0</t>
+          <t>69.0</t>
         </is>
       </c>
       <c r="AC15" s="2" t="inlineStr">
         <is>
-          <t>1/10</t>
+          <t>3/10</t>
         </is>
       </c>
     </row>
@@ -2246,32 +2270,36 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>全程车</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>09:28</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>73分钟</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr"/>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="inlineStr"/>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
           <t>06:02</t>
@@ -2279,7 +2307,7 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -2303,29 +2331,29 @@
       </c>
       <c r="W16" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X16" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y16" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z16" s="2" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA16" s="2" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="AA16" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="AB16" s="2" t="inlineStr">
         <is>
           <t>73.0</t>
@@ -2333,7 +2361,7 @@
       </c>
       <c r="AC16" s="2" t="inlineStr">
         <is>
-          <t>5/10</t>
+          <t>6/10</t>
         </is>
       </c>
     </row>
@@ -2394,7 +2422,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -2509,7 +2537,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
@@ -2548,7 +2576,7 @@
       </c>
       <c r="Z18" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="AA18" s="2" t="inlineStr">
@@ -2620,7 +2648,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -2674,7 +2702,7 @@
       </c>
       <c r="AC19" s="2" t="inlineStr">
         <is>
-          <t>6/10</t>
+          <t>7/10</t>
         </is>
       </c>
     </row>
@@ -2735,7 +2763,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2846,7 +2874,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
@@ -2890,13 +2918,17 @@
       </c>
       <c r="AA21" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB21" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB21" s="2" t="inlineStr">
+        <is>
+          <t>68.0</t>
+        </is>
+      </c>
       <c r="AC21" s="2" t="inlineStr">
         <is>
-          <t>—/10</t>
+          <t>1/10</t>
         </is>
       </c>
     </row>
@@ -2904,22 +2936,22 @@
       <c r="A22" s="2" t="inlineStr"/>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>沪A55712D</t>
+          <t>沪A67353D</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
           <t>川沙客运站</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>09:18</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>金杨路金口路</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -2952,12 +2984,12 @@
       <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="inlineStr">
         <is>
-          <t>06:02</t>
+          <t>07:11</t>
         </is>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -2971,47 +3003,618 @@
       <c r="T22" s="2" t="inlineStr"/>
       <c r="U22" s="2" t="inlineStr">
         <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="V22" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W22" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X22" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y22" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z22" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA22" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB22" s="2" t="inlineStr">
+        <is>
+          <t>75.0</t>
+        </is>
+      </c>
+      <c r="AC22" s="2" t="inlineStr">
+        <is>
+          <t>8/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr"/>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>沪A55712D</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
           <t>09:18</t>
         </is>
       </c>
-      <c r="V22" s="2" t="inlineStr">
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr"/>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>09:11</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q23" s="2" t="inlineStr"/>
+      <c r="R23" s="2" t="inlineStr"/>
+      <c r="S23" s="2" t="inlineStr"/>
+      <c r="T23" s="2" t="inlineStr"/>
+      <c r="U23" s="2" t="inlineStr">
+        <is>
+          <t>09:18</t>
+        </is>
+      </c>
+      <c r="V23" s="2" t="inlineStr">
         <is>
           <t>计划发车</t>
         </is>
       </c>
-      <c r="W22" s="2" t="inlineStr">
+      <c r="W23" s="2" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="X22" s="2" t="inlineStr">
-        <is>
-          <t>待确认</t>
-        </is>
-      </c>
-      <c r="Y22" s="2" t="inlineStr">
+      <c r="X23" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y23" s="2" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="Z22" s="2" t="inlineStr">
+      <c r="Z23" s="2" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="AA22" s="2" t="inlineStr">
+      <c r="AA23" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AB22" s="2" t="inlineStr">
+      <c r="AB23" s="2" t="inlineStr">
         <is>
           <t>72.0</t>
         </is>
       </c>
-      <c r="AC22" s="2" t="inlineStr">
-        <is>
-          <t>4/10</t>
+      <c r="AC23" s="2" t="inlineStr">
+        <is>
+          <t>5/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr"/>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>沪A66513D</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr"/>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>09:11</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q24" s="2" t="inlineStr"/>
+      <c r="R24" s="2" t="inlineStr"/>
+      <c r="S24" s="2" t="inlineStr"/>
+      <c r="T24" s="2" t="inlineStr"/>
+      <c r="U24" s="2" t="inlineStr">
+        <is>
+          <t>09:35</t>
+        </is>
+      </c>
+      <c r="V24" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W24" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X24" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y24" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z24" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA24" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB24" s="2" t="inlineStr">
+        <is>
+          <t>69.0</t>
+        </is>
+      </c>
+      <c r="AC24" s="2" t="inlineStr">
+        <is>
+          <t>3/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr"/>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>沪A67026D</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>09:46</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr"/>
+      <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr"/>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>09:11</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q25" s="2" t="inlineStr"/>
+      <c r="R25" s="2" t="inlineStr"/>
+      <c r="S25" s="2" t="inlineStr"/>
+      <c r="T25" s="2" t="inlineStr"/>
+      <c r="U25" s="2" t="inlineStr">
+        <is>
+          <t>09:46</t>
+        </is>
+      </c>
+      <c r="V25" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W25" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X25" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y25" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z25" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA25" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB25" s="2" t="inlineStr">
+        <is>
+          <t>69.0</t>
+        </is>
+      </c>
+      <c r="AC25" s="2" t="inlineStr">
+        <is>
+          <t>3/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr"/>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>沪A32298D</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr"/>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>09:11</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q26" s="2" t="inlineStr"/>
+      <c r="R26" s="2" t="inlineStr"/>
+      <c r="S26" s="2" t="inlineStr"/>
+      <c r="T26" s="2" t="inlineStr"/>
+      <c r="U26" s="2" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="V26" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W26" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X26" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y26" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z26" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA26" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AB26" s="2" t="inlineStr"/>
+      <c r="AC26" s="2" t="inlineStr">
+        <is>
+          <t>—/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr"/>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>沪A67983D</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>10:14</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>既无可靠终点到达证据，也未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr"/>
+      <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr"/>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>06:02</t>
+        </is>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>09:11</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q27" s="2" t="inlineStr"/>
+      <c r="R27" s="2" t="inlineStr"/>
+      <c r="S27" s="2" t="inlineStr"/>
+      <c r="T27" s="2" t="inlineStr"/>
+      <c r="U27" s="2" t="inlineStr">
+        <is>
+          <t>10:14</t>
+        </is>
+      </c>
+      <c r="V27" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W27" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X27" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="Y27" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z27" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="AA27" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB27" s="2" t="inlineStr">
+        <is>
+          <t>73.0</t>
+        </is>
+      </c>
+      <c r="AC27" s="2" t="inlineStr">
+        <is>
+          <t>6/10</t>
         </is>
       </c>
     </row>

</xml_diff>